<commit_message>
Categorize the 27 previously-uncategorized lectures
Assigned each to Foundations in Bhakti (kept philosophy/guru/principles) or
Festivals and Kirtans (kirtan/holy-name/festival/sankirtana talks: wk28,30,45,67,80).
Updated manifest, spreadsheet Category column, note front-matter, CATEGORIES.md
(now Foundations 46 / Festivals 33), and the README lecture index. No lecture
is uncategorized. Also refreshed two stale README lines for the structured-notes format.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/Pre-Initiation_IDS_course_modules.xlsx
+++ b/build/Pre-Initiation_IDS_course_modules.xlsx
@@ -643,6 +643,11 @@
           <t>Speaking on Bhagavad-gita 9.27-28, Indradyumna Swami explains Krishna consciousness as 'the art of all work': any action performed separately from Krishna's service plants a seed of karma, but action whose fruits are offered to Krishna (yukta-vairagya, as described by Rupa Goswami) burns up these seeds and clears the mirror of the mind. He stresses that even so-called good material activity causes bondage, quoting Krishnadas Kaviraj Goswami of the Chaitanya-caritamrita that there is nothing truly good in this world because everything is temporary and ends in suffering, even on the heavenly planets. He reframes the disciplines of sadhana-bhakti as 'the regulative principles of freedom': the non-devotee is a helpless slave of mind and senses (material nature as Rudrani, 'she who makes you cry forever'), while the devotee freely chooses to serve Krishna and is therefore liberated even now, since he follows the instructions of a liberated spiritual master. Prabhupada's mood of 'work now, samadhi later' and the supreme value of preaching and book distribution (sankirtan) are emphasized as the highest taste, following the example of Chaitanya Mahaprabhu and Srila Prabhupada. He illustrates the liberated devotee's detachment with the lotus flower that grows in water yet never touches it. In the concluding Q&amp;A he tells the story of Surya Narayan, a materialistic Spanish banker who blasphemed and had a book-distributing devotee arrested in Paris, then read the discarded Krishna books, gradually surrendered, and became a first-class devotee and temple treasurer in Barcelona, showing the unlimited delivering potency of Lord Chaitanya's mercy.</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G6" s="11" t="n"/>
       <c r="H6" s="11" t="n"/>
       <c r="I6" s="11" t="n"/>
@@ -888,6 +893,11 @@
           <t>[Not summarized — detected pl]</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G11" s="11" t="n"/>
       <c r="H11" s="11" t="n"/>
       <c r="I11" s="11" t="n"/>
@@ -933,6 +943,11 @@
           <t>Indradyumna Swami offers a Srila Prabhupada glorification composed entirely of personal reminiscences from the early 1970s, beginning with first seeing Srila Prabhupada at the Detroit airport in 1971, where devotees wept while he, a new devotee, worried he was too materially attached to cry, and where Prabhupada's words 'you are not this body' pierced his heart. He recounts his eight-month wait for initiation, giving his emergency ten dollars to the Bhaktivedanta Book Fund with a letter, and receiving a reply promising that Prabhupada would in due course accept him as a duly initiated disciple. He tells of arranging to fly with Prabhupada to Europe, confronting a rude customs officer over Prabhupada's white bag, walking alone with Prabhupada who three times explained that people in the material world have no good qualities because of the modes of nature but recover them by reviving Krishna consciousness, honoring orange-peel maha-prasadam on the plane, and watching a Charlie Chaplin film that Prabhupada justified because 'Krishna is the origin of all original things.' Further stories cover being left behind in London to carry Prabhupada's heavy bag of Acharya commentaries and receiving the blessing 'so much endeavor in this material world, but when I take you back to Godhead everything will be easy and sublime,' plus receiving one of Prabhupada's dhotis with the instruction to 'preach boldly and have faith in the holy names.' In France he describes the poor Paris temple, the installation of Radha Paris-Ishvara where Prabhupada lovingly treated the marble Deity as directly Radharani, drinking all the charanamrita after winning a book-distribution marathon, and seeing Prabhupada shed torrents of tears while singing 'Jaya Radha-Madhava' in separation from Krishna. He relates preaching to and converting a French Navy admiral (told to read the ninth chapter of the Bhagavad-gita) and the transformation of a filthy, drug-addicted homeless boy nicknamed 'Pigpen' whom Prabhupada blessed with 'it's all right, my boy,' and who became the initiated book distributor Rasada Das. The talk closes on Prabhupada as the perfect gentleman and expert preacher who could touch any heart, redirecting a woman's question from her past life to her next, yet who could also thunder in righteous anger 'you are not God, you are a dog' when Krishna was blasphemed.</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G12" s="11" t="n"/>
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="11" t="n"/>
@@ -976,6 +991,11 @@
       <c r="E13" s="19" t="inlineStr">
         <is>
           <t>Lecturing from Sri Chaitanya-caritamrita (Madhya-lila) at New Raman Reti (Alachua), Indradyumna Swami examines Rupa and Sanatana Goswamis' famous expression of humility — calling themselves lower than the sinners Jagai and Madhai for having associated with meat-eaters while serving in the government of the Muslim ruler Hussain Shah. Though they are eternally liberated associates of Radharani (Rupa Manjari and Rati/Lavanga Manjari), they display the crown-jewel Vaishnava quality of humility to teach conditioned souls the danger of bad association. Retelling how Sanatana was pressed into service as chief minister, he stresses the power of association — good or bad — since we take on the qualities of those we associate with, like a chameleon. He speaks strongly against meat-eating: it is violence (himsa), it implicates the eater in a conspiracy of slaughter, and Sri Isopanisad calls a meat-eater atma-ha, "killer of the soul" — not killing the soul itself but killing its opportunity for self-realization. Yet, like bell-metal turned to gold, even the most fallen can be transformed into a brahmana and Vaishnava through chanting and initiation. Through Prahlada Maharaja's prayer he warns that a devotee's only real fear is forgetting Krishna's lotus feet under maya's influence, and that the shelter — like crabs fleeing into the vast ocean, or taking refuge in Krishna — is the association of devotees, which Prabhupada created ISKCON to provide. Ending "on a high note," he affirms that anyone's destiny can be changed in the association of the Lord and His devotees.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
         </is>
       </c>
     </row>
@@ -1120,6 +1140,11 @@
           <t>Speaking on Bhagavad-gita 15.7, Indradyumna Swami establishes the true identity of the living entity as an eternal fragmental part and parcel of Krishna, qualitatively one with God (like sun rays sharing the sun's qualities) but not quantitatively equal, and eternally a servant of the Lord. Under the illusion of maya, which both covers reality and drives the soul away from Krishna, the living entity falsely identifies with the gross material body through ahankara (false ego), the strongest material element that survives even death and, as he says, nuclear war. Because of this bodily identification the soul struggles with the six senses and the mind, suffering repeated birth, death, old age, and disease, and searches for happiness in the wrong place. The remedy is transcendental knowledge received from a bona fide spiritual master, who removes the cataract of ignorance like a surgeon's scalpel and plants the seed of devotional service (bhakti-lata-bija) in the disciple's heart through his instructions. This seed is watered by hearing and chanting (sravanam kirtanam), so that dormant love of God, latent within everyone like the kingdom of God within, is awakened by the transcendental sound of the Hare Krishna maha-mantra. Swami stresses the simple, scientific process of hearing about Krishna, chanting Hare Krishna, and honoring prasadam, which cleanses the heart of all material desire, and concludes that the goal of all philosophy is to bring one to surrender and loving service under the guidance of a self-realized soul.</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G3" s="11" t="n"/>
       <c r="H3" s="11" t="n"/>
       <c r="I3" s="11" t="n"/>
@@ -1165,6 +1190,11 @@
           <t>Taking Bhagavad-gita 2.11 as his text, Indradyumna Swami reflects on Krishna's opening the Gita by indirectly calling Arjuna a fool, and how a genuine disciple welcomes such chastisement just as a patient is relieved when a doctor finally names the disease. He argues that we are all in fact fools, because we exchanged an eternal life of bliss and knowledge in loving relationship with Krishna for a temporary material life of ignorance and suffering, a trade he likens to swapping a 500-Deutschmark note for a single mark. Real intelligence, he says, is knowing one is a fool and approaching a bona fide spiritual master with humility, illustrated by Sanatana Goswami putting grass between his lips before Chaitanya Mahaprabhu and admitting that despite all his learning he did not know who he is. Because material qualifications can actually obstruct devotion (like a violin student's ingrained bad habits, and as Kunti Devi prays), what attracts Krishna is not opulence but sincere love, shown by Prabhupada's delight at a poor sweeper woman's rose over a businessman's thousand-dollar check. The Swami stresses that the truly urgent problems are birth, disease, old age, and death, so the human form and its youthful vigor should be used now for Krishna consciousness, retelling Bhaktisiddhanta Saraswati's story of the man hanging in a well, ignoring the rope of the guru's mercy to lick more drops of sense-gratification honey. He explains that the guru must teach both matter and spirit, that Krishna is bhakta-vatsala (partial to His devotees, not to jnanis, yogis, or sense-enjoyers), and that constant association with Krishna, as enjoyed by the Vrindavan residents and Pandavas, comes only through pure devotion free of lust, anger, and greed. In the Q&amp;A he teaches that only a submissive hearer can be convinced (through the Gita's philosophy or the higher taste of chanting and prasadam, Lord Chaitanya's "secret weapon"), and that one may trust a bona fide representative who follows the guru's instructions exactly. He closes by framing his modest gathering as the budding of a great preaching tour, citing the Durban festival attended by Nelson Mandela and the Polish Woodstock preaching as evidence that a pure devotee's "dreams" are simply reality awaiting its time to manifest.</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G4" s="11" t="n"/>
       <c r="H4" s="11" t="n"/>
       <c r="I4" s="11" t="n"/>
@@ -1610,6 +1640,11 @@
           <t>Speaking on the Caitanya-caritamrta chapter 'The Lord Tastes Nectar' — which recounts Krishna's confidential pastimes with the gopis that Lord Caitanya relished for eighteen years at Jagannatha Puri in his Antya-lila — Indradyumna Swami explains that neophyte devotees should hear these wholly transcendental pastimes as purifying medicine rather than try to imitate or enter them prematurely. He repeatedly warns against sahajiya cheating (taking devotion cheaply, enjoying the Lord's intimate lilas while still attached to sense gratification), illustrated by the Bengali image of a horse that tries to eat grass while jumping and by Prabhupada rebuking disciples who visit Radha-kunda without being able to follow even the first verse of the Upadeshamrta. The heart of the talk is Prabhupada's instruction to see with 'a good eye and a bad eye': a preacher and Prabhupada's purports reveal two things at once — the face of Maya (the material world seen for the misery it is) and the face of Krishna — so that hearing of Krishna's sweetness awakens a strong hankering for Him instead of envy of materialists. Swami stresses that devotees are not missing anything now, being already surrounded by Krishna's mercy in the holy name, guru, deities, prasada and books, and that the path is 'perfect, more perfect, most perfect,' nectar 'from the word go.' He teaches that the four regulative principles are not austerities but simply giving up suffering, and that the process, though simple, is not cheap — one must throw off the 'sandbags' of attachment, as a hot-air balloon must, to rise. Through many stories — fool's gold in the Sierra Nevadas, a child's bicycle training wheels representing Guru and Gauranga, Prabhupada offering a chain-smoking life member the 'special mercy' of losing everything, and Narada and Shiva relishing a fragment of Krishna's prasada — he shows that devotional service is more powerful than God Himself and is freely bestowed by the magnanimous Lord Caitanya, though it must be received by paying the price of full surrender, with guru-shastra-sadhu as one's balance.</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G13" s="11" t="n"/>
       <c r="H13" s="11" t="n"/>
       <c r="I13" s="11" t="n"/>
@@ -1655,6 +1690,11 @@
           <t>Indradyumna Swami presents the 'essence of Bhagavad-gita' to a largely new audience, first establishing that Krishna consciousness is not some newly-invented Eastern religion but one of the oldest spiritual traditions, at least 5,000 years old and authoritative because it rests on scripture spoken by God Himself. He explains that religion (from the Latin religio, 'to reconnect with God') is neither Eastern nor Western, and that just as one teacher teaches mathematics differently to first-graders and to university students, God has revealed different scriptures according to time, place and people's capacity, with the Gita being the 'PhD on the science of self-realization.' Taking the question 'Who am I?', he teaches that we are not the material body but the spark of life within it; the body is only a sophisticated machine (yantra) that, like a Mac computer or a Toyota, is useless without the conscious soul who drives it, and the soul (per BG 2.20) is never born and never dies. He then explains death and reincarnation: as the soul passes from a child's body to youth to old age (and as the body renews every seven years), at death it passes into one of 8,400,000 species according to the desires and consciousness it has cultivated, and life is present from conception because only living things grow. He warns that seeking happiness in this world is illusion (maya, 'that which is not') — like a man hunting for his lost keys under a streetlight merely because the light is better, or reaching for apples reflected in water and getting only a mouthful — a perverted reflection of the soul's own intrinsically blissful (sat-cit-ananda) nature, which is as natural to it as sweetness to sugar or wetness to water. Because the material world is temporary and full of suffering while the spiritual world is eternal and full of bliss, and because spiritual advancement (unlike the wealth the Egyptians vainly buried with their kings) is carried forward into the next life, one should invest this human life in self-realization by hearing from self-realized souls. Acknowledging that modern people have no time for forest meditation or elaborate rituals, he offers the special concession for the age of Kali: chanting the Hare Krishna maha-mantra, since the holy name is non-different from God and awards the 'higher taste' that lets one naturally give up intoxication, illicit sex and gambling. He closes by inviting everyone to test the process and judge it by its result (phalena pariciyate), then leads the audience in chanting.</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G14" s="11" t="n"/>
       <c r="H14" s="11" t="n"/>
       <c r="I14" s="11" t="n"/>
@@ -1700,7 +1740,11 @@
           <t>Speaking at a temple 'Festival of Appreciation,' Indradyumna Swami takes up Prahlada Maharaja's prayer from the Seventh Canto of Srimad Bhagavatam, in which Prahlada rejects material opulence, liberation, and mystic perfection (bhukti, mukti, siddhi) and begs only to be placed in the service of a pure devotee, using it to explain why appreciating and associating with devotees is central to Krishna consciousness. He teaches that Krishna decorates his surrendered devotees with all good qualities and places them in prominent positions so ordinary people will recognize and follow them, comparing this to war heroes honored with medals after World War II. Drawing on the verse titiksavah karunikah (SB 3.25.21), he describes the genuine devotee as tolerant even in calamity, compassionate (compassion being the crest-jewel of Vaishnava qualities), and a friend to every living being with no enemies, because he sees everyone's original nature as an eternal servant of Krishna. Because we are the Lord's tiny marginal energy (tatastha-shakti), we take on the qualities of whatever we associate with, like a chameleon, so bad association, including the subtle 'one-eyed guru' of television, music, and idle talk, can quickly drag down even great souls (illustrated by Ajamila, the tortoise and the hare, and swine flu), while a single moment's association with a devotee can award all success and transmit bhakti like a contagious 'good disease.' The secret for devotees living among materialists, he says, is to give association rather than take it. He then summarizes the five most potent limbs of devotion, associating with devotees, chanting the holy name, hearing the Bhagavatam, residing in Mathura, and worshiping the deity, arguing that association of devotees is the 'salt' that brings out the flavor and result of all the others, since chanting must be learned through initiation from a bona fide guru and the Bhagavatam heard from a living 'person-bhagavata,' not merely read. He urges the devotees to recognize and serve the advanced Vaishnavas present in this fleeting generation, honoring every devotee's service great or small (like the tiny screw that holds a harmonium together and the 'silent soldiers' behind the feast). He closes by having everyone fold their hands and recite the Vaishnava-pranama prayer to honor all the Vaishnavas present and throughout the world.</t>
         </is>
       </c>
-      <c r="F15" s="11" t="n"/>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G15" s="11" t="n"/>
       <c r="H15" s="11" t="n"/>
       <c r="I15" s="11" t="n"/>
@@ -1746,6 +1790,11 @@
           <t>Speaking on Bhagavad-gita 10.36 - where Krishna declares 'I am the gambling of cheats, the splendor of the splendid, victory, adventure, and the strength of the strong' - Indradyumna Swami fixes on the phrase 'I am adventure' to show how the natural human craving for excitement can be dovetailed in Krishna's service. He argues that the material world, from the highest planet to the lowest, is temporary and full of misery, a place of repeated birth and death (BG 8.15-16), so it is no true venue for adventure; real happiness comes only when the soul returns to its natural position as Krishna's eternal servant and offers everything to Him with love (BG 9.26-27, SB 1.2.6). Krishna Himself is 'adventurous,' descending from Vaikuntha to deliver the pious and vanquish demons (BG 4.8), and devotees join that adventure by spreading Krishna consciousness despite opposition, trusting the Lord's protection (BG 9.22; the Bengali saying 'rakhe Krishna mare ke, mare Krishna rakhe ke'; the example of Prahlada). The Swami illustrates all this with vivid autobiographical stories: his restless American youth (surfer, Marine Corps, disillusionment with the Vietnam war) redirected by Srila Prabhupada into the adventure of preaching; a brahmachari Sankirtan party in Marseille menaced first by a Hell's Angels motorcycle gang and then by gypsies, resolved by claiming brotherhood, chanting the Nrisimha prayer, and marching boldly forward, with the whole gypsy village finally routing the bikers; and a border crossing into war-torn Dagestan where he and his companions, mistaken for Indian 'mullahs,' led 10,000 Muslims at a wedding in chanting the Hare Krishna maha-mantra as praise of Allah. He stresses that these are the modern-day pastimes of Lord Chaitanya, that the guru's instruction carries with it the power to execute it, and that prasadam and the holy name soften even the hardest hearts (agyata-sukriti - unknowing devotional service is still accepted by the Lord). He closes with a call - echoing Lord Chaitanya's instruction to those born in Bharat (CC Madhya 9.41) - for Indians to reclaim their fading spiritual culture, purify themselves by chanting, and take up the real adventure of saving the world, since human life is meant first for self-realization (Vedanta-sutra: athato brahma-jijnasa).</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Festivals and Kirtans</t>
+        </is>
+      </c>
       <c r="G16" s="11" t="n"/>
       <c r="H16" s="11" t="n"/>
       <c r="I16" s="11" t="n"/>
@@ -1839,6 +1888,11 @@
       <c r="E18" s="19" t="inlineStr">
         <is>
           <t>In 1987 Indradyumna Swami was invited to preach Krishna consciousness in Brazil, and after touring all 37 temples of the successful Brazilian yatra he became determined to carry the sankirtana movement into the remote Amazon jungle. Flying to the tiny preaching center in Manaus, where nine devotees had not seen another devotee in two and a half years, he found they had no money and no boat, the only means of jungle travel, so he prayed to Lord Chaitanya for a way to go. At a Sunday feast he met a heavyset, aristocratic woman who turned out to be the wife of the state governor; calling herself only 'a tiny servant of Krishna,' she miraculously arranged the governor's own palatial white riverboat with a seven-man crew, 2,000 US dollars for fuel, a ton of grains, and months of provisions, even drawing her pistol to make the crew agree to become vegetarian. Traveling up the Amazon past alligators, piranha, and giant piraiba fish, the devotees overcame their fear and held kirtan for isolated tribal villagers, who danced, chanted 'Haribol,' took prasadam, and thought the white-skinned devotees were gods from heaven; Maharaja explained who Krishna is by narrating the pastime of Aghasura, the giant serpent demon Krishna killed in Vrindavan. Because the simple people could not accept the four regulative principles, he preached only chanting the holy name, and after each program the villagers wept and begged them to stay, the chief kneeling and saying they wanted to change their lives and live like the devotees. Over roughly two months they visited some 60 to 70 villages and distributed about 65,000 plates of khichari and many books, surviving poisonous moths, snakes, a near-fatal bout of dysentery cured overnight by a jungle medicine man, a quicksand trap in a swamp full of alligators, and a hurricane-like storm. On the return journey even the boat's captain, who had taken prasadam for two months including Mahaprasadam of Lord Nrisimhadeva, spontaneously proclaimed 'All glories to the sankirtana movement of Lord Chaitanya Mahaprabhu' and remained vegetarian two years later, while the governor's wife met them joyfully at the Manaus dock, insisting there had been 'no problems' because Krishna had brought them safely back. Maharaja concludes that the story reveals the unstoppable power of Lord Chaitanya's mercy, which can transform even the lowest of people, and that with determination and enthusiasm devotees can preach and distribute books to anyone.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Festivals and Kirtans</t>
         </is>
       </c>
       <c r="G18" s="11" t="n"/>
@@ -2509,7 +2563,11 @@
           <t>Speaking in Calcutta on the eve of 2025, Indradyumna Swami addresses the theme of New Year's resolutions, observing that December 31st is a Western import absent from the Vaishnava calendar: the Vedic new year falls on the first day of Chaitra (April/May) and the Gaudiya new year on Gaura Purnima, Lord Chaitanya's appearance day. He warns against 'watering down' the tradition by adding foreign observances, illustrating the danger with Prabhupada's 'cat in the basket' story, in which one lady's accidental act hardens over generations into a false 'Vedic tradition.' The best way to spend the evening, he says, is in kirtan, since not even a moment should be wasted away from remembrance of Krishna; noting that only nine percent of Americans keep their resolutions, he jokes that Vaishnavas need make no new vows at all, because they have already taken the supreme resolution to serve Krishna, like Hanuman's firm and unshaken vow to serve Rama. Because love is reciprocal, Krishna reciprocates a sincere vow, just as Rama vows to award fearlessness to anyone who surrenders even once, and the Avanti brahmana's resolution to cross the ocean of nescience by serving Krishna's lotus feet bears fruit not through formal sannyasa but through chanting the holy name. He urges strict adherence to the four vows already taken (no meat-eating, intoxication, illicit sex, or gambling), comparing them to Bhishma's 'terrible vow,' and explains they are sustainable only through the higher taste of chanting, per Chanakya Pandit's maxim that one gives up something only for something better. He traces how Lord Chaitanya's strictness was progressively made accessible by Bhaktisiddhanta Saraswati and then Prabhupada, recalling Prabhupada's three-and-a-half-hour kirtan in Tompkins Square Park, the purifying potency of transcendental sound (shabda-brahma) even when the language is not understood, and prasadam as Chaitanya's 'secret weapon' (the Notre Dame priest and the dripping gulab-jamun in Paris). He closes by urging devotees to keep the goal of prema (pure love of God) constantly in view, using his boyhood Disneyland trip as an analogy, to avoid procrastination (Prahlada rebuking his young playmates), and to reaffirm and increase the quality of their existing vows, chanting more than the minimum sixteen rounds and studying Prabhupada's books, rather than inventing trivial new ones.</t>
         </is>
       </c>
-      <c r="F13" s="11" t="n"/>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G13" s="11" t="n"/>
       <c r="H13" s="11" t="n"/>
       <c r="I13" s="11" t="n"/>
@@ -2555,6 +2613,11 @@
           <t>Speaking on the theme of controlling versus engaging the senses (rooted in Prahlada Maharaja's warning in Srimad Bhagavatam 7.5.30 that persons of uncontrolled senses glide toward hell, endlessly 'chewing the chewed'), Indradyumna Swami argues that spiritual life is not merely negating the senses but re-engaging them in Krishna's devotional service. He contrasts this with the impersonalist (Mayavadi) error of trying to kill desire: desire cannot be killed, only purified and redirected to the Lord. Through the story of Narada Muni's cobra disciple (told not to bite but still allowed to hiss and scare, like a snake with its fangs removed) and a story of Jesus curing a disciple's tapeworm by ordering twenty days of fasting and then forbidding him to drink warm saffron-honey milk, he shows that the guru's restrictions and seemingly impossible tests exist to purify the disciple, even when the instruction is not understood. He warns that sense gratification breeds an 'I, me and mine' mentality that hardens the heart and turns to fault-finding and criticizing devotees, which is the first offense to the holy name; a real Vaishnava first sees a devotee's service and only then his faults, just as a hospital is full of sick people who are nonetheless there to become well. The remedy is humility (thinking oneself lower than a blade of grass), gratitude (readiness to say 'thank you' and 'I'm sorry'), and the reciprocal exchange of gifts, which he illustrates with his own back-and-forth of gifts with a congregation member who repaired his car. He stresses full faith in and surrender to the spiritual master, never wanting to embarrass the guru who recommends the disciple to Krishna, and recalls his own first contact with Vishnujana Swami and other sannyasis and his early longing for the devotees. Finally he teaches that freedom from envy and material desire produces the compassion needed for effective preaching, as the Six Goswamis attracted even rogues because they came only to give and not to take; since the only thing that can stop the movement is the internal enemy of material desire, the conclusion is that 'books are the basis, preaching is the essence, utility is the principle, and purity is the force' - so when asked the best preaching technique, the best thing is purity.</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G14" s="11" t="n"/>
       <c r="H14" s="11" t="n"/>
       <c r="I14" s="11" t="n"/>
@@ -2596,7 +2659,11 @@
           <t>[Not summarized — detected ru]</t>
         </is>
       </c>
-      <c r="F15" s="11" t="n"/>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G15" s="11" t="n"/>
       <c r="H15" s="11" t="n"/>
       <c r="I15" s="11" t="n"/>
@@ -2642,6 +2709,11 @@
           <t>This is an introductory address given by Indradyumna Swami before a public kirtan at a Festival of India program in Poland. He explains that kirtan means glorifying God by singing His holy names, and that although there is only one God, He is known by different names in different languages, just as the one sun is called by different names around the world; in India that name is Krishna, meaning the most attractive and most beautiful person. Because God is absolute, he stresses, the Lord is fully present in the sound of His name, so that unlike the material world where saying 'water, water, water' cannot quench one's thirst since the name and the object are different, chanting 'Hare Krishna' actually gives one direct association with the Supreme Lord. He teaches that all living beings once lived with God in the spiritual world and, having come to the material world, foolishly seek lasting happiness in temporary material things that are here today and gone tomorrow, when what they truly hanker for is the happiness of God's association. Correcting the common Western image of God as old, grey-haired and feeble, he cites the Vedic description of God as simultaneously the oldest person and the father of creation, yet eternally youthful, with a spiritual, ever-blissful body. Observing that everyone, whatever their differences, agrees on wanting to be happy, he says the Vedic scriptures recommend congregational chanting of the holy name as the easiest and most sublime means of awakening love of God in this age. Using the analogy that Poles love pizza even though it came from Italy, he explains that although chanting arose in India it is meant for everyone, since all souls are part of God's family rather than merely Polish, German, American or Japanese, and that this transcendental sound never becomes tiresome even after chanting for thirty or forty years, unlike material radio songs, because it touches and awakens the soul. He closes by teaching the audience the Hare Krishna maha-mantra so they can chant along and experience the same joy.</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Festivals and Kirtans</t>
+        </is>
+      </c>
       <c r="G16" s="11" t="n"/>
       <c r="H16" s="11" t="n"/>
       <c r="I16" s="11" t="n"/>
@@ -2687,6 +2759,11 @@
           <t>Delivered on the appearance day of Srila Narottama dasa Thakura, this lecture glorifies him as a rare acharya who was simultaneously a perfect bhajananandi (deep rasika devotee) and a perfect goshthyanandi (preacher), likening him to Haridasa Thakura whom Chaitanya Mahaprabhu praised for both practicing and preaching purely, and noting that Narottama's works Prarthana and Prema-bhakti-candrika are treasured as good as, or better than, Veda because he is nitya-siddha. Maharaja recounts how Chaitanya Mahaprabhu, during sankirtana at Ramakeli, ecstatically foretold Narottama's appearance and entrusted liquid prema-bhakti to the personified Padma River (Padmavati) to hold until Narottama should bathe in her waters. He narrates Narottama's life: his birth to King Krishnananda Datta and Narayani, the astrologer's warning that he must never bathe in a river, his infant refusal of unoffered sweet rice, and the roughly twelve years he spent hearing Chaitanya's pastimes until Nityananda appeared in a dream directing him to the Padma, where Padmavati poured prema over him, his body erupted in the eight ecstatic symptoms, and he turned golden like Mahaprabhu. The heart of the talk is guru-nishta, faith in and attachment to the spiritual master: obeying the Lord's dream-order, Narottama abandons his kingdom, walks barefoot through the jungle to Vrindavan only to learn Rupa and Sanatana had just departed, and then wins initiation from the reluctant Lokanatha Goswami through determined, humble menial service, secretly cleaning the spot where his would-be guru passed stool until the old acharya's heart melts. Maharaja weaves in humility as the crest-jewel of devotional qualities and the ideal of desiring only service birth after birth, not wealth, followers, women, or a GBC/guru/sannyasi position. Under Jiva Goswami at the Radha-Damodara temple Narottama advances so rapidly in manasa-seva that, absorbed as the gopi Vilasa Manjari minding Champakalata's boiling milk for Krishna, he actually burns his physical hands. Finally titled and empowered, he receives Lokanatha's two parting instructions, to always serve the deity and always spread Mahaprabhu's sankirtana, is sent with the Goswamis' books toward Bengal, and at Navadvipa is embraced and blessed by the departed associates of the Lord to rejuvenate the movement, the lecture dwelling throughout on the sweetness of vipralambha (separation) as the highest wealth of devotion.</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G17" s="11" t="n"/>
       <c r="H17" s="11" t="n"/>
       <c r="I17" s="11" t="n"/>
@@ -2732,6 +2809,11 @@
           <t>Delivered as an arrival address at Indradyumna Swami's Polish festival tour, this talk centers on cultivating a genuine service attitude as the foundation of Vaishnava relationships. The speaker, freshly returned from the Montreal and Toronto Rathayatra festivals, recalls being moved by the ecstatic dancing of the Hare Krishna Youth Bus Tour, where even a passing sixteen-year-old girl began to weep on seeing the devotees' joyful life. Echoing Srila Prabhupada's saying that 'one who has life can preach,' he praises the vitality of the festival and muses that the Polish tour could one day grow into Prabhupada's dream of an international, world-traveling sankirtan party. Accepting the warm reception offered to him, he stresses that Vaishnava culture is built on respecting devotees, and that a tragic failing in society is when devotees lose respect for one another. His central thesis is that respect can only be preserved through a constant service attitude: rendering service to more advanced devotees, preaching together with equals as close friends, and creating facilities for less advanced devotees to serve, so that one always thinks 'I am the servant of everyone.' He contrasts this Vaishnava mood with the Mayavadi sannyasi who imagines 'I am Narayana,' and illustrates it with the story of Sarvabhauma Bhattacharya and Chaitanya Mahaprabhu at Jagannatha Puri. In the question-and-answer portion he explains that busy, service-filled engagement leaves 'no time' to lose respect, that only those with too much idle time manufacture reasons for conflict, and that even envy is killed at the root by rendering service, humorously demonstrating this with a prasadam-serving anecdote.</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G18" s="11" t="n"/>
       <c r="H18" s="11" t="n"/>
       <c r="I18" s="11" t="n"/>
@@ -2777,6 +2859,11 @@
           <t>Delivered before an initiation ceremony, Indradyumna Swami explains that initiation is the formal beginning of spiritual life, in which the candidates vow to chant sixteen rounds daily, follow the four regulative principles, and serve Guru and Gauranga. He compares initiation to a binding legal contract between two serious parties: the disciple promises to follow the regulative process of bhajana-kriya, while the spiritual master accepts full responsibility to deliver the disciple, even being prepared to take birth again if necessary, though the disciple should live so as to spare the guru that trouble. Using a story of rescuing a drowning, panicking girl in Mexico when he was sixteen, he teaches that a disciple should make the guru's work easy by fully surrendering the past rather than clinging to material conditioning. He explains why the name is changed at initiation, comparing it to a bride leaving her father's family, and stresses that our only true identity is as the eternal servant of Krishna, so a Vaishnava should never be judged by his bodily or national conditioning (illustrated by the spotted moon that still gives light and flavor to vegetables). He notes the day is especially auspicious because it is when Raghunatha dasa Goswami received the mercy of Lord Nityananda, and he narrates that pastime at length: Raghunatha's wealthy parents guarded him and married him to a beautiful chaste girl to keep him home, yet he prayed only to be delivered from the ditch of material life. At the Panihati festival, Nityananda placed His lotus feet on Raghunatha's head and ordered him to feed the Vaishnavas with chipped rice and yogurt, a festival Lord Chaitanya Himself attended; when Raghunatha begged for pure devotion (not wealth, followers, beauty, or even liberation), his desire was fulfilled and he later escaped his guarded home through the help of his initiating guru Yadunandana Acharya to reach Chaitanya Mahaprabhu, who placed him under Svarupa Damodara. The Swami concludes that this potent day embodies the very spirit of initiation: approaching the representative of the guru-parampara with humility and surrendering one's life to Hari, Guru, and Vaishnavas.</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G19" s="11" t="n"/>
       <c r="H19" s="11" t="n"/>
       <c r="I19" s="11" t="n"/>
@@ -2822,6 +2909,11 @@
           <t>Speaking at an initiation ceremony in Dallas (eight devotees receiving first initiation and eight receiving second), Indradyumna Swami builds his talk on Srimad Bhagavatam 7.9.28, where Prahlada Maharaja, offered any benediction by the Lord, instead begs to keep serving his spiritual master Narada Muni. This shows the central principle that one must first serve and please the guru, through whose mercy the seed of devotion (bhakti-lata-bija) is awakened and Krishna's mercy then follows. He describes initiation as a second, spiritual birth, contrasting it with ordinary birth, which is into ignorance because the soul abandoned Krishna and the eternal spiritual world for the temporary, suffering material world, likened to Durga-dham, a prison walled in by birth, disease, old age, and death, with the material body as the prisoner's uniform. The seed of bhakti lies dormant in every heart until the guru activates it and authorizes the disciple to chant Hare Krishna; chanting even before initiation frees one from sin and material desire, but attaining prema, pure love of God, requires receiving the mantra in bona fide disciplic succession. Because a genuine brahmana cannot tolerate the pain of material existence, he seeks a solution and takes shelter of a spiritual master, holding onto the guru's lotus feet, inquiring submissively and applying his instructions (pariprasnena sevaya). Meeting such a sadhu is extremely rare, and in Kali-yuga the guru mercifully comes to find the fallen soul, as Srila Prabhupada came to the West. The most essential instruction is the chanting of the holy name, which the Swami calls Kali-yuga's special mercy, a permanent sale of the holy name that yields in this age what meditation, sacrifice, and temple worship gave in previous ages. He closes by urging the initiates never to lose sight of the goal, the day when a tear of love for Krishna flows down the cheek, quoting Rupa Goswami that the holy names create a jubilant festival in the mouth and material desires no longer appear beautiful.</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G20" s="11" t="n"/>
       <c r="H20" s="11" t="n"/>
       <c r="I20" s="11" t="n"/>
@@ -2865,6 +2957,11 @@
       <c r="E21" s="19" t="inlineStr">
         <is>
           <t>Speaking on a spring afternoon in Budapest, Indradyumna Swami lectures on Bhagavad-gita 18.55, teaching that Krishna can be understood only through pure devotional service under the guidance of a pure devotee, not by scholarship or mental speculation, and that such full devotion carries the soul back into the kingdom of God. He traces the soul's fall from the spiritual world through envy: the Lord accompanies and pleads with the departing soul, and though we imagine ourselves independent (like a bull tied to a post by his nose-rope), we remain forever dependent, placed under the charge of Maya/Durga, who binds us with the ropes of the three gunas and, as our stern 'foster mother' (Rudrani, 'she who makes you cry'), torments us precisely so we will turn back to God. He drives home the certainty of death with a personal story of a melanoma scare in Durban that briefly gave him a six-month prognosis, showing how the so-called beauty of this world instantly faded and only the lotus feet of Radha and Krishna remained important. Since the soul's intrinsic nature is to serve Krishna (as the hand serves the stomach), material 'happiness' is merely temporary relief from suffering, and the cure for a despondent devotee is to get up and resume service. The whole purpose of the creation is to frustrate us until we turn our face from the shadow back toward God's effulgent form, so everyone is eventually brought to their knees, whether by good intelligence (recognizing that the order in creation, from atom to universe, implies a supreme intelligence) or by death, as in the story of Khrushchev's cosmonaut who denied God until his craft burned up crying 'Oh my God, please help me.' Krishna, seated in every heart as the Supersoul and truest friend, hears the sincere cry and guides the soul to the association of devotees and to a bona fide spiritual master, the external manifestation of the Supersoul who both blesses and, being 'heavy' (guru), chastises. Yet the Maharaja's central point is that we must 'do our part': like a life-preserver thrown to a drowning man, Krishna's mercy must be seized and held tight through chanting, hearing, dancing, taking prasadam and visiting holy places, for though the Lord does most of the pulling, Mother Yashoda still had to add her own 'one inch' of effort to bind baby Krishna.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
         </is>
       </c>
       <c r="G21" s="11" t="n"/>
@@ -3617,7 +3714,11 @@
           <t>In this London disciple meeting (a "warm-up" Vyasa Puja), Indradyumna Swami reassures his disciples that his reduced visits stem not from displeasure but from expanding responsibilities. He explains that chanting Hare Krishna is more a heartfelt prayer for service than a mechanical mantra, and that although our worldly masters have been merciless, serving Hari, Guru, and the Vaishnavas — a merciful master — reveals the real joy of service (illustrated by Prabhupada's example of the well-kept dog with a master versus the suffering strays). Growing responsibility, he says, is a sign the process is working, just as a father entrusts the family business to a mature son, and as the Lord entrusts His mission only to His most intimate servants. He recounts how, while contemplating retirement to a simple bhajan life in India, a prayer to Lord Shiva at Ujjain inspired him to bring the festival tour to India to help preserve Vedic culture — yet loving letters from his disciples reminded him not to serve one part of his mission at the expense of another. He closes by promising to remain a steadfast lighthouse for his disciples, always available, and to keep returning every year.</t>
         </is>
       </c>
-      <c r="F14" s="11" t="n"/>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G14" s="11" t="n"/>
       <c r="H14" s="11" t="n"/>
       <c r="I14" s="11" t="n"/>
@@ -3663,6 +3764,11 @@
           <t>His Holiness Indradyumna Swami explains that one may approach Krishna even while full of material desires, because the association itself purifies—just as a blind man who cannot appreciate fire still benefits from its warmth. Citing Srimad-Bhagavatam 2.3.10, he says that whether one is desireless, full of material desire, or seeking liberation, one should worship the Supreme Lord, which is why even an offensive chanter of the holy name can still be purified if his desire is sincere. The goal, however, is to advance past material motivation to a higher taste (Bhagavad-gita 2.59), giving up sense gratification rather than clutching both—illustrated by Dhruva Maharaja, who after seeing the Lord regarded his hard-won kingdom as a mere pebble beside a diamond, and by the monkey that trapped its own hand by refusing to release a banana. Quoting Prabhupada's purport, he stresses that 'sense gratification and Krishna consciousness go ill together,' like oil and water that never mix. The devotee must therefore mature out of the childish 'give me, give me' stage—which the father and the spiritual master tolerate for a time—into nishtha, the steady stage of unmotivated, uninterrupted devotional service (Srimad-Bhagavatam 1.2.6), becoming responsible and a shelter for other devotees instead of lamenting a lack of association. He contrasts complaining, well-facilitated devotees with the young, persecuted devotees in Russia who have no temple and read scripture in dark rooms yet still go out to preach. The temple, Prabhupada said, is not a place for eating and sleeping but a base for preaching; one should take only what is necessary (Sri Isopanishad, mantra 1) and offer the balance in service, ultimately reaching desirelessness (nishkama) and following the gopis, who—as Prabhupada wept to recall—never asked anything of Krishna but only wished to please Him, which is the very definition of pure devotion (Bhakti-rasamrita-sindhu 1.1.11). In the question period he adds that material facility is safe only when supervised by guru and Krishna, that one need not remember past misdeeds to surrender now (the drowning man who should board the boat rather than ask questions), and that Jaya and Vijaya fell to the material world to satisfy the Lord's own desire for combat.</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G15" s="11" t="n"/>
       <c r="H15" s="11" t="n"/>
       <c r="I15" s="11" t="n"/>
@@ -3704,6 +3810,11 @@
           <t>Speaking on Srimad Bhagavatam 5.18.13 (Canto 5, Chapter 18, 'The Residents of Jambudvipa Offer Prayers'), Indradyumna Swami explains that just as aquatics thrive only in vast water, the living entity manifests its full glory only in relationship with the Supreme Lord as His eternal servant (jivera svarupa haya krishna nitya dasa), while a soul cut off from that connection becomes weak and insignificant, like a crocodile fierce in water but helpless and awkward on land. He illustrates the point with a chain of homely analogies: Prabhupada's beach dogs in Bombay (fat and cared-for when they have a master, skinny strays when they run away), a beautiful peach flower that withers the moment it is picked from the tree, a screw or a thumb that is essential in place but disgusting once separated, and a heart taken out of the body during a triple-bypass operation and kept alive only by artificial machines, showing that material existence is merely 'artificial life' whereas real life is devotional service. He warns that the material energy is 'maximum security prison' of birth, death, old age and disease which even yogis and jnanis cannot escape (Bhagavad-gita 7.14), and that greatness by material calculation is momentary and humiliating in old age, citing Johnny Weissmuller (Tarzan) and Elvis Presley whose very bodily assets became sources of their downfall. He teaches yukta-vairagya, real renunciation, meaning to use everything in Krishna's service rather than falsely giving it up as the Mayavadis do, quoting Bhaktivinoda Thakura who saw his large family and home transformed into Vaikuntha, and stresses the great strength gained through celibacy and controlled senses, with Bhaktisiddhanta Saraswati as the example of a naisthika-brahmachari of extraordinary memory and preaching power. The core thesis is that our strength lies in our strictness: the real hero is not the athlete but the one who controls his mind and senses and keeps his initiation vows without compromise, since compromise is 'Maya's last trick.' He drives this home with the vows of Arjuna (rejecting Urvasi as his mother, and going into exile to keep the Pandavas' agreement over Draupadi), Bhishma's lifelong brahmacharya vow for his father Shantanu, and Prabhupada's simple rebuke 'but you promised.' He closes with Abhimanyu, who learned how to enter the military formation but not how to get out, to warn that we must accept and apply every instruction of the spiritual master, not just the prominent ones, encouraged by Bhaktisiddhanta Saraswati's assurance that all his disciples could go back to Godhead in this very lifetime if they remain strict.</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G16" s="11" t="n"/>
       <c r="H16" s="11" t="n"/>
       <c r="I16" s="11" t="n"/>
@@ -3749,6 +3860,11 @@
           <t>Speaking to a university audience at an ISKCON festival, Indradyumna Swami introduces the philosophy of the Bhagavad Gita, presenting it not as a new religion but as one of humanity's oldest spiritual traditions and an 'unabridged spiritual dictionary' that can answer any question about spiritual life. His core theme is that the human form, uniquely endowed with intelligence (buddhi), is the rare chance to inquire into the self ('athato brahma jijnasa') and to act on it now. He argues that we are not the material body (yantra, a machine) but the eternal soul (atma) that drives it, contrasting a whole life spent 'polishing the car' with neglecting the driver inside, and explains transmigration of the soul, karma, and the spiritual equality of all living beings. This equality grounds his case for vegetarianism, which he illustrates with the story of how, as a fourteen-year-old football and swim-team captain, a single visit to a slaughterhouse arranged by his vegetarian father made him give up meat on the spot. He describes the material world as a temporary place of duality and suffering, a 'prison' where even Bill Gates cannot escape birth, disease, old age and death, and names mukti (liberation), the return to a loving relationship with a personal God, as life's real goal. The practical process he recommends is chanting the Hare Krishna maha-mantra, which awakens the sleeping soul like an alarm clock, supported by a disciplined daily life (rising in the brahma-muhurta, sixteen rounds of japa on 108 beads, Bhagavad Gita study) and four regulative principles: no meat, no intoxication, no illicit sex, and no gambling. In the extended Q&amp;A he explains that vegetarianism is completed by offering food to Krishna as prasadam (making it karma-free), defends the need for a bona fide guru as God's empowered representative (a 'telescope' that brings the distant moon near), and clarifies that self-realization is not merging into an impersonal void but reawakening one of several eternal loving relationships (rasa) with God, as servant, friend, parent, or lover.</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G17" s="11" t="n"/>
       <c r="H17" s="11" t="n"/>
       <c r="I17" s="11" t="n"/>
@@ -3792,6 +3908,11 @@
       <c r="E18" s="19" t="inlineStr">
         <is>
           <t>Delivered on the day of the Panihati (Chipped Rice) Festival, this lecture by Indradyumna Swami reads from the Chaitanya-caritamrita the pastime in which Nityananda Prabhu playfully calls the wealthy young Raghunath Das a 'thief' and 'punishes' him by ordering a feast of chipped rice and yogurt for all the devotees on the bank of the Ganges near Panihati. Indradyumna Swami uses Raghunath Das Goswami's life to illustrate genuine renunciation: because he possessed the highest thing (attachment to Radha-Krishna and Lord Chaitanya), he could easily abandon his wealth, wife, and comforts, following the niti-sastra logic that 'you can only give up something if you get something better.' He stresses that devotees need not imitate artificial austerities; renunciation comes naturally by chanting Hare Krishna, honoring prasadam, hearing Srimad-Bhagavatam, and serving devotees, with unwanted desires falling away like a snake's shed skin as one matures, though pratistha (the subtle desire for honor) is the hardest impurity to remove. Turning to the goal, he identifies Raghunath Das Goswami as the 'prayojana guru' who reveals the highest attainment: pure love of God (prema) in the mood of the gopis of Vraja, and especially love in separation (vipralambha), which is described as more relishable than meeting Krishna. Reading through the Shikshashtaka, Prabhupada's letters, and the Nectar of Devotion, he teaches that one should learn to cry for the Lord and hanker for that goal even while practicing the basics. He recounts the pastime of Advaita Acharya, whose tears of love Mahaprabhu 'locked in a knot' on his japa rope so that he could keep managing and preaching, to show that prema is sometimes withheld from preachers whose service the mission still needs. The central exhortation, echoing Prabhupada's plan for an 18-day Mahabharata film in Nairobi, is to 'think big': faithfully do one's daily service now, but aspire boldly to go back to Godhead, where the spiritual master takes the disciple's hand and places it in Krishna's.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Festivals and Kirtans</t>
         </is>
       </c>
       <c r="G18" s="11" t="n"/>
@@ -4213,6 +4334,11 @@
           <t>Continuing his series on Srila Narottama Das Thakura, Indradyumna Swami recounts how, after the historic first Gaura-purnima festival at Kheturi, Narottama and his intimate companion Ramachandra Kaviraja (described as one soul in two bodies) began preaching Lord Chaitanya's message in earnest, meeting fierce opposition from caste brahmanas who resented that Narottama, a Kayastha by birth, was initiating brahmanas. Through a series of dramatic conversions he transformed his opponents: a proud karma-kandi brahmana afflicted with leprosy was cured limb by limb while dancing in Narottama's kirtan; two goatherd boys, Hari Rama and Ramakrishna, bound for a Durga sacrifice, overheard the two Vaishnavas loudly discussing philosophy, freed their animals, and became empowered preachers who, with the king's physician Balaram, defeated the undefeated debater (digvijaya) Murari; and the learned brahmana Ganga Narayan Chakravarti surrendered after Narottama appeared to him in a dream. When hundreds of brahmanas led by Rupa Narayan and King Narasingha marched on Kheturi to defeat him, Narottama's disciples, disguised as a betel-nut seller and a clay-pot seller, defeated the pundits in Sanskrit, and Durga herself appeared in the brahmanas' dreams affirming Krishna's supremacy and demanding their surrender. The speaker dwells at length on the dacoit-king Hari Chandarai, who, tortured from within by a Brahmana-rakshasa ghost, was freed by Narottama's mere glance; after becoming a fixed chanter of the holy name he was imprisoned in a filthy pit and condemned to execution by a maddened elephant by a vengeful Yavana king, but, praying to his guru, he seized the charging elephant's trunk and killed it, melting the king's heart, and afterward converted whole bands of dacoits. Narottama's mission spread even to tribal Manipur, whose king (converted by Ganga Narayan) decreed universal Vaishnavism, and Indradyumna Swami interweaves personal reminiscences of Srila Prabhupada's glance, a stoning by Maoist youths at a modern Manipur festival, and a practical letter of Vishvanatha Chakravarti Thakura found in the Jaipur archives asking the king to protect pilgrims from dacoits. The lecture closes with Narottama's overwhelming separation on learning of the deaths of Ramachandra Kaviraja and Srinivasa Acharya, during which he composed his famous song of separation from the Vaishnavas; his own passing on a funeral pyre, from which he miraculously returned to life bearing a shining sacred thread to save the blaspheming brahmanas at Ganga Narayan's compassionate plea; and his final disappearance, when his body melted into milk in the Ganges, leaving the humble Dudh (milk) Samadhi, after which he twice reappeared amid the mourners' kirtan to console every Vaishnava and promise he would always be with them.</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Foundations in Bhakti</t>
+        </is>
+      </c>
       <c r="G8" s="11" t="n"/>
       <c r="H8" s="11" t="n"/>
       <c r="I8" s="11" t="n"/>
@@ -4456,6 +4582,11 @@
       <c r="E13" s="19" t="inlineStr">
         <is>
           <t>Speaking at a festival themed 'Dance to the Source of the Love' (Krishna), Indradyumna Swami first honors his godbrother Radhanath Swami for pioneering preaching to leaders and the higher echelon of society, recalling how Srila Prabhupada in Paris repeatedly asked the sankirtana devotees to 'bring some intelligent people for me to preach to,' and beamed when they produced a professor, author, poet, politician and rock star. He shares his own formative memory of Prabhupada instructing him, as he left for France, to 'preach boldly and have faith in the holy names,' and gifting him a used dhoti with the words that a gift from a Vaishnava is very special. The heart of the talk is the potency of transcendental sound: he explains that 'by sound one becomes conditioned and by sound one becomes liberated,' illustrating with a radio dial that shifts the heart from sad blues to happy songs to angry news, then contrasting this with the maha-mantra which descends from Goloka and awakens prema. He unpacks 'mantra' as that which delivers the mind from the bodily concept of life, notes that in past ages only qualified brahmanas could chant effectively while Kali-yuga offers the concession that anyone may chant the holy name as the yuga-dharma, and tells the story of Ramanujacharya, who broadcast his guru's secret mantra from atop a pole so that everyone could be delivered, embodying the compassionate Vaishnava heart. Citing Shukadeva Goswami's teaching that although Kali-yuga is an ocean of inauspiciousness its one good quality is that chanting Krishna's names grants liberation, he stresses that the holy name is non-different from God and is itself His incarnation. He warns that without understanding the glories and philosophy of the name we chant like a child who swallows a diamond ring unaware of its value, recommends studying the BBT's Namamrita, and relays Prabhupada rendering the mantra to a Boston boy as simply 'my friend, my friend, my friend'-a desperate prayer of the heart. He closes with a South Africa story: on a violently windy, twice-aborted landing at Durban's La Mercy airport, passengers of every faith cried out to God, and a skeptic beside him who dismissed it as 'sentimental rubbish' was finally persuaded to chant 'Hare Krishna'; when the wind died and the plane landed, the man moved from atheist to agnostic, proving to Maharaja that God is present in the sound of His name.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Festivals and Kirtans</t>
         </is>
       </c>
       <c r="G13" s="11" t="n"/>

</xml_diff>